<commit_message>
add: Boa parte das extrações dos dados dos portais já foram feitas, falta Leroy e Pluri; o que está funcional aparentemente está gerando tudo corretamente
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -47,25 +47,25 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>BRUNO NASCIMENTO JACONELLI</t>
-  </si>
-  <si>
-    <t>427.771.148-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policlinica capao raso </t>
-  </si>
-  <si>
-    <t>G43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marcio Duarte Coutinho </t>
+    <t>JULIANO CEZAR ZANARDI</t>
+  </si>
+  <si>
+    <t>064.324.839-05</t>
+  </si>
+  <si>
+    <t>Hospital São Lucas</t>
+  </si>
+  <si>
+    <t>M54.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sylvio José Palu </t>
   </si>
   <si>
     <t>PR</t>
   </si>
   <si>
-    <t>23104</t>
+    <t>12.555</t>
   </si>
 </sst>
 </file>
@@ -442,14 +442,14 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="31.706543" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="25.85083" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="28.135986" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="21.137695" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="7">
-        <v>45903</v>
+        <v>45932</v>
       </c>
       <c r="E2" s="8">
         <v>1</v>

</xml_diff>

<commit_message>
fix & add: conserto de bugs gerais de execução, refatoração de código e mudança de estrutura de diretórios; adição da centralização das credenciais num unico arquivos
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,25 +47,13 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>JULIANO CEZAR ZANARDI</t>
-  </si>
-  <si>
-    <t>064.324.839-05</t>
-  </si>
-  <si>
-    <t>Hospital São Lucas</t>
-  </si>
-  <si>
-    <t>M54.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sylvio José Palu </t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>12.555</t>
+    <t>JULIANA DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>000.975.920-48</t>
+  </si>
+  <si>
+    <t>RS</t>
   </si>
 </sst>
 </file>
@@ -442,14 +430,14 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="25.85083" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="28.135986" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="21.137695" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="17.567139" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -495,26 +483,18 @@
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="7">
-        <v>45932</v>
+        <v>45931</v>
       </c>
       <c r="E2" s="8">
         <v>1</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="J2" s="3"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
add: extração de dados da pluri e leroy funcional, tratamento e formatação dos dados ainda não 100% configurados
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,10 +47,13 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>RICHARD GRAMM QUADRADO</t>
-  </si>
-  <si>
-    <t>049.184.340-29</t>
+    <t>JOSE AUGUSTO VITER ALVES</t>
+  </si>
+  <si>
+    <t>037.469.479-60</t>
+  </si>
+  <si>
+    <t>IMA</t>
   </si>
 </sst>
 </file>
@@ -422,7 +425,7 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="26.993408" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="29.421387" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
@@ -478,7 +481,9 @@
       <c r="E2" s="7">
         <v>0</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>

</xml_diff>

<commit_message>
fix: lógica de start_date e end_date ajustada e outros ajustes
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,20 +47,34 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>JOSE AUGUSTO VITER ALVES</t>
-  </si>
-  <si>
-    <t>037.469.479-60</t>
-  </si>
-  <si>
-    <t>IMA</t>
+    <t>RAMON MAISCK BRAGA</t>
+  </si>
+  <si>
+    <t>050.112.405-50</t>
+  </si>
+  <si>
+    <t>HOSPITAL TERESA DE LISIEUX</t>
+  </si>
+  <si>
+    <t>M779</t>
+  </si>
+  <si>
+    <t>FABIO RODRIGUES DE LIMA</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>CRM - 16742</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <b val="0"/>
@@ -98,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -118,6 +132,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
@@ -425,14 +442,14 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="29.421387" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="17.567139" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="28.135986" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -477,17 +494,27 @@
         <v>11</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="7">
-        <v>0</v>
+      <c r="D2" s="7">
+        <v>45936</v>
+      </c>
+      <c r="E2" s="8">
+        <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
fix: Resolvido problema de falha de interação com o DOM: responsavilidade estava causando problema, foi ajustado pra o browser sempre maximizar o tamanho da janela
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,34 +47,29 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>RAMON MAISCK BRAGA</t>
-  </si>
-  <si>
-    <t>050.112.405-50</t>
-  </si>
-  <si>
-    <t>HOSPITAL TERESA DE LISIEUX</t>
-  </si>
-  <si>
-    <t>M779</t>
-  </si>
-  <si>
-    <t>FABIO RODRIGUES DE LIMA</t>
-  </si>
-  <si>
-    <t>BA</t>
-  </si>
-  <si>
-    <t>CRM - 16742</t>
+    <t>GUILHERME DE SOUSA</t>
+  </si>
+  <si>
+    <t>103.257.287-63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consulta médica </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingrind Schmidt tagomori </t>
+  </si>
+  <si>
+    <t>RJ</t>
+  </si>
+  <si>
+    <t>5247648-8p</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <b val="0"/>
@@ -112,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -132,9 +127,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
@@ -449,7 +441,7 @@
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="28.135986" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="30.563965" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -494,26 +486,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="7">
-        <v>45936</v>
-      </c>
-      <c r="E2" s="8">
+      <c r="D2" s="5"/>
+      <c r="E2" s="7">
         <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add: adição da Viva e outras mudanças
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,22 +47,10 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>GUILHERME DE SOUSA</t>
-  </si>
-  <si>
-    <t>103.257.287-63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consulta médica </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingrind Schmidt tagomori </t>
-  </si>
-  <si>
-    <t>RJ</t>
-  </si>
-  <si>
-    <t>5247648-8p</t>
+    <t>DAVID FERREIRA DE SOUZA</t>
+  </si>
+  <si>
+    <t>924.800.399-00</t>
   </si>
 </sst>
 </file>
@@ -434,14 +422,14 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="22.280273" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="28.135986" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="30.563965" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="17.567139" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -490,19 +478,11 @@
       <c r="E2" s="7">
         <v>1</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
fix: Algumas mudanças no salvamento dos arquivos
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,34 +47,29 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>RAMON MAISCK BRAGA</t>
-  </si>
-  <si>
-    <t>050.112.405-50</t>
-  </si>
-  <si>
-    <t>HOSPITAL TERESA DE LISIEUX</t>
-  </si>
-  <si>
-    <t>M779</t>
-  </si>
-  <si>
-    <t>FABIO RODRIGUES DE LIMA</t>
-  </si>
-  <si>
-    <t>BA</t>
-  </si>
-  <si>
-    <t>CRM - 16742</t>
+    <t>GUILHERME DE SOUSA</t>
+  </si>
+  <si>
+    <t>103.257.287-63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consulta médica </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingrind Schmidt tagomori </t>
+  </si>
+  <si>
+    <t>RJ</t>
+  </si>
+  <si>
+    <t>5247648-8p</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <b val="0"/>
@@ -112,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -132,9 +127,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
@@ -449,7 +441,7 @@
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="28.135986" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="30.563965" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -494,26 +486,22 @@
         <v>11</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="7">
-        <v>45936</v>
-      </c>
-      <c r="E2" s="8">
+      <c r="D2" s="5"/>
+      <c r="E2" s="7">
         <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: alterado nome de pasta da pluri e outras pequenas mudanças
</commit_message>
<xml_diff>
--- a/data/greif/temp/grid_db_suporte (1).xlsx
+++ b/data/greif/temp/grid_db_suporte (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
   <si>
     <t>Cod Funcionario</t>
   </si>
@@ -47,29 +47,34 @@
     <t>Atestado Crm</t>
   </si>
   <si>
-    <t>GUILHERME DE SOUSA</t>
-  </si>
-  <si>
-    <t>103.257.287-63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consulta médica </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingrind Schmidt tagomori </t>
-  </si>
-  <si>
-    <t>RJ</t>
-  </si>
-  <si>
-    <t>5247648-8p</t>
+    <t>EVERTON LUIZ RODRIGUES DOS SANTOS</t>
+  </si>
+  <si>
+    <t>041.655.219-65</t>
+  </si>
+  <si>
+    <t>Concemed Centro médico e diagnóstico</t>
+  </si>
+  <si>
+    <t>M 545</t>
+  </si>
+  <si>
+    <t>Dra Carolina Nascimento</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>CRM-43470</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <b val="0"/>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -127,6 +132,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1">
@@ -434,14 +442,14 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="22.280273" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="39.990234" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711426" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="24.708252" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="22.280273" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="62.41333" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="30.563965" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="28.135986" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="8.140869" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="15.281982" bestFit="true" customWidth="true" style="0"/>
   </cols>
@@ -486,22 +494,26 @@
         <v>11</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="7">
+      <c r="D2" s="7">
+        <v>45945</v>
+      </c>
+      <c r="E2" s="8">
         <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3"/>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="H2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>